<commit_message>
Refresh state-wise overdue data from praapti.in (as of 2026-10-12)
Re-scraped home/getStateWiseOverdueReport. National totals now:
Current 64,059.9 Cr, Overdue Before Trigger 22,576.5 Cr,
Overdue After Trigger 6.4 Cr (portal last updated 2026-10-11).
State list unchanged at 33 states/UTs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QDkN6JmvLtVVBxV7MZ6VWz
</commit_message>
<xml_diff>
--- a/Praapti_StateWise_Overdue.xlsx
+++ b/Praapti_StateWise_Overdue.xlsx
@@ -520,7 +520,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: https://praapti.in (home/getStateWiseOverdueReport)  |  All amounts in Rs. Crore  |  Scraped: 2026-09-09</t>
+          <t>Source: https://praapti.in (home/getStateWiseOverdueReport)  |  All amounts in Rs. Crore  |  Scraped: 2026-10-12</t>
         </is>
       </c>
     </row>
@@ -573,16 +573,16 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>3361.3710722</v>
+        <v>3208.199778</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2709.6378901</v>
+        <v>3390.4153886</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>2709.6378901</v>
+        <v>3390.4153886</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
@@ -602,16 +602,16 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>47.8955964</v>
+        <v>47.9222487</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>0.6029133</v>
+        <v>0</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>0.0005735</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>0.6034868</v>
+        <v>0.0005735</v>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
@@ -631,16 +631,16 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1360.5232556</v>
+        <v>1204.8927087</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>35.7164126</v>
+        <v>105.609945</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>0.4617117</v>
+        <v>0.9716452</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>36.1781243</v>
+        <v>106.5815902</v>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
@@ -660,16 +660,16 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>3887.1073671</v>
+        <v>3854.7991369</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>727.6239772</v>
+        <v>1523.4736275</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.1536194</v>
+        <v>0.3072388</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>727.7775966</v>
+        <v>1523.7808663</v>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
@@ -689,16 +689,16 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>201.2615955</v>
+        <v>126.649349</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>5.0556505</v>
+        <v>5.404365</v>
       </c>
       <c r="E9" s="6" t="n">
         <v>0.0040492</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>5.0596997</v>
+        <v>5.4084142</v>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
@@ -718,16 +718,16 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>2268.8155338</v>
+        <v>1666.4715944</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>66.2599251</v>
+        <v>63.8003176</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>0.047929</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>66.3078541</v>
+        <v>63.8482466</v>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
@@ -747,20 +747,20 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>729.3385638</v>
+        <v>718.9311396000001</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>1.7721306</v>
+        <v>0</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>1.7721306</v>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Overdue Before Trigger Date</t>
+        <v>0</v>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Current dues</t>
         </is>
       </c>
     </row>
@@ -776,16 +776,16 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>1814.746618</v>
+        <v>1863.9337604</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>117.5293895</v>
+        <v>299.3949728</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>0.7150193</v>
+        <v>0.8237261</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>118.2444088</v>
+        <v>300.2186989</v>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
@@ -805,16 +805,16 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>87.06176550000001</v>
+        <v>53.4731628</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>1.0048546</v>
+        <v>0.9838589</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>1.0048546</v>
+        <v>0.9838589</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
@@ -834,16 +834,16 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2884.7720937</v>
+        <v>3079.1626909</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>119.8052713</v>
+        <v>354.1750921</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>9e-07</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>119.8052722</v>
+        <v>354.175093</v>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
@@ -863,16 +863,16 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>3382.6870038</v>
+        <v>3400.3072011</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1410.8557868</v>
+        <v>937.9660574</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>3e-07</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>1410.8557871</v>
+        <v>937.9660577</v>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
@@ -892,16 +892,16 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>423.7210428</v>
+        <v>411.2619116</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>36.4218143</v>
+        <v>43.0692083</v>
       </c>
       <c r="E16" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>36.4218143</v>
+        <v>43.0692083</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
@@ -921,20 +921,20 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>1307.5120904</v>
+        <v>1104.0779979</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0</v>
+        <v>0.0681266</v>
       </c>
       <c r="E17" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>Current dues</t>
+        <v>0.0681266</v>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
@@ -950,16 +950,16 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>1987.785782</v>
+        <v>1919.4936329</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>30.9451448</v>
+        <v>479.0766011</v>
       </c>
       <c r="E18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>30.9451448</v>
+        <v>479.0766011</v>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
@@ -979,16 +979,16 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>4847.3128162</v>
+        <v>4937.7810923</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>2801.3576706</v>
+        <v>2453.4638587</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1.8787265</v>
+        <v>2.453557</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>2803.2363971</v>
+        <v>2455.9174157</v>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
@@ -1008,16 +1008,16 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>773.3769996</v>
+        <v>1382.9556319</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>32.9250338</v>
+        <v>149.7663968</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.1701943</v>
+        <v>0.2421294</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>33.0952281</v>
+        <v>150.0085262</v>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
@@ -1037,16 +1037,16 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>2976.5197561</v>
+        <v>3894.0066592</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>865.6462972</v>
+        <v>193.2048152</v>
       </c>
       <c r="E21" s="6" t="n">
         <v>0.0178909</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>865.6641881</v>
+        <v>193.2227061</v>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
@@ -1066,16 +1066,16 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>6161.2741929</v>
+        <v>5860.0466961</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>2298.2043696</v>
+        <v>2288.5244573</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.5829442</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>2298.7873138</v>
+        <v>2289.1074015</v>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
@@ -1095,20 +1095,20 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>145.051854</v>
+        <v>131.731206</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>42.151892</v>
+        <v>70.99196209999999</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0</v>
+        <v>0.0446027</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>42.151892</v>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Overdue Before Trigger Date</t>
+        <v>71.03656479999999</v>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Overdue After Trigger Date</t>
         </is>
       </c>
     </row>
@@ -1124,20 +1124,20 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>80.4057152</v>
+        <v>83.52207610000001</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>2.9477522</v>
+        <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>2.9477522</v>
-      </c>
-      <c r="G24" s="7" t="inlineStr">
-        <is>
-          <t>Overdue Before Trigger Date</t>
+        <v>0</v>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>Current dues</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>41.0678718</v>
+        <v>54.5828016</v>
       </c>
       <c r="D25" s="6" t="n">
         <v>0</v>
@@ -1182,20 +1182,20 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>65.5716819</v>
+        <v>100.094225</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0</v>
+        <v>13.7237376</v>
       </c>
       <c r="E26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>Current dues</t>
+        <v>13.7237376</v>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Overdue Before Trigger Date</t>
         </is>
       </c>
     </row>
@@ -1211,16 +1211,16 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>1300.287625</v>
+        <v>1408.7929364</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>474.0948632</v>
+        <v>408.2612053</v>
       </c>
       <c r="E27" s="6" t="n">
         <v>0.2621178</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>474.356981</v>
+        <v>408.5233231</v>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
@@ -1240,16 +1240,16 @@
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>290.6929106</v>
+        <v>310.4932153</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>28.2946496</v>
+        <v>64.47586509999999</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>28.2946496</v>
+        <v>64.47586509999999</v>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
@@ -1269,16 +1269,16 @@
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>3249.4679334</v>
+        <v>3048.5868092</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>414.4290736</v>
+        <v>398.2184799</v>
       </c>
       <c r="E29" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>414.4290736</v>
+        <v>398.2184799</v>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
@@ -1298,16 +1298,16 @@
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>4382.8169765</v>
+        <v>3993.483277</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>2440.8323243</v>
+        <v>2788.2409008</v>
       </c>
       <c r="E30" s="6" t="n">
         <v>0.009858799999999999</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>2440.8421831</v>
+        <v>2788.2507596</v>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
@@ -1327,16 +1327,16 @@
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>52.0196783</v>
+        <v>56.2528851</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>31.001355</v>
+        <v>22.7576671</v>
       </c>
       <c r="E31" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>31.001355</v>
+        <v>22.7576671</v>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
@@ -1356,16 +1356,16 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>2915.8491</v>
+        <v>3933.7231966</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>849.8763079</v>
+        <v>1775.5807606</v>
       </c>
       <c r="E32" s="6" t="n">
         <v>2e-07</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>849.8763081</v>
+        <v>1775.5807608</v>
       </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
@@ -1385,16 +1385,16 @@
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>1582.8874538</v>
+        <v>1648.1299255</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>69.7638122</v>
+        <v>113.3299422</v>
       </c>
       <c r="E33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>69.7638122</v>
+        <v>113.3299422</v>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
@@ -1414,16 +1414,16 @@
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>307.6319081</v>
+        <v>284.567492</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>215.8977762</v>
+        <v>193.0120572</v>
       </c>
       <c r="E34" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>215.8977762</v>
+        <v>193.0120572</v>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
@@ -1443,16 +1443,16 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>8681.8565652</v>
+        <v>7820.0122814</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>5592.5716273</v>
+        <v>3875.1090739</v>
       </c>
       <c r="E35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>5592.5716273</v>
+        <v>3875.1090739</v>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
@@ -1472,16 +1472,16 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>842.2709733</v>
+        <v>752.8084711</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>143.9289141</v>
+        <v>101.8059567</v>
       </c>
       <c r="E36" s="6" t="n">
         <v>0.2664035</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>144.1953176</v>
+        <v>102.0723602</v>
       </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
@@ -1501,16 +1501,16 @@
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>1608.4779702</v>
+        <v>1698.7330907</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>189.6500489</v>
+        <v>462.5719473</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>0.3530568</v>
+        <v>0.3601519</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>190.0031057</v>
+        <v>462.9320992</v>
       </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
@@ -1526,16 +1526,16 @@
       </c>
       <c r="B38" s="11" t="n"/>
       <c r="C38" s="12" t="n">
-        <v>64049.4393627</v>
+        <v>64059.88028139999</v>
       </c>
       <c r="D38" s="12" t="n">
-        <v>21756.8049284</v>
+        <v>22576.4766447</v>
       </c>
       <c r="E38" s="12" t="n">
-        <v>4.9240963</v>
+        <v>6.3948194</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>21761.7290247</v>
+        <v>22582.8714641</v>
       </c>
       <c r="G38" s="11" t="n"/>
     </row>

</xml_diff>